<commit_message>
Update ETF provider exports and extractor fixes
</commit_message>
<xml_diff>
--- a/providers/invesco/2026-07-06/invesco_etf_export.xlsx
+++ b/providers/invesco/2026-07-06/invesco_etf_export.xlsx
@@ -376,10 +376,10 @@
         <v>0.1</v>
       </c>
       <c r="G9">
-        <v>23197516.65</v>
+        <v>23194958.23</v>
       </c>
       <c r="H9">
-        <v>5.8665</v>
+        <v>5.86706</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -417,10 +417,10 @@
         <v>0.1</v>
       </c>
       <c r="G10">
-        <v>23197516.65</v>
+        <v>23194958.23</v>
       </c>
       <c r="H10">
-        <v>5.33309</v>
+        <v>5.3336</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -458,10 +458,10 @@
         <v>0.12</v>
       </c>
       <c r="G11">
-        <v>17345883.014917567</v>
+        <v>17343969.96298651</v>
       </c>
       <c r="H11">
-        <v>5.86514</v>
+        <v>5.86571</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -499,10 +499,10 @@
         <v>0.12</v>
       </c>
       <c r="G12">
-        <v>17345883.014917567</v>
+        <v>17343969.96298651</v>
       </c>
       <c r="H12">
-        <v>5.35104</v>
+        <v>5.3516</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -622,10 +622,10 @@
         <v>0.1</v>
       </c>
       <c r="G15">
-        <v>15302670.57</v>
+        <v>15299312.76</v>
       </c>
       <c r="H15">
-        <v>5.8396</v>
+        <v>5.84021</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -663,10 +663,10 @@
         <v>0.1</v>
       </c>
       <c r="G16">
-        <v>15302670.57</v>
+        <v>15299312.76</v>
       </c>
       <c r="H16">
-        <v>5.31604</v>
+        <v>5.31659</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -704,10 +704,10 @@
         <v>0.12</v>
       </c>
       <c r="G17">
-        <v>11442532.29894942</v>
+        <v>11440021.505215542</v>
       </c>
       <c r="H17">
-        <v>5.83495</v>
+        <v>5.83561</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -745,10 +745,10 @@
         <v>0.12</v>
       </c>
       <c r="G18">
-        <v>11442532.29894942</v>
+        <v>11440021.505215542</v>
       </c>
       <c r="H18">
-        <v>5.33049</v>
+        <v>5.33107</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -868,10 +868,10 @@
         <v>0.1</v>
       </c>
       <c r="G21">
-        <v>30402541.99</v>
+        <v>30400022.22</v>
       </c>
       <c r="H21">
-        <v>5.80274</v>
+        <v>5.80339</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -909,10 +909,10 @@
         <v>0.1</v>
       </c>
       <c r="G22">
-        <v>30402541.99</v>
+        <v>30400022.22</v>
       </c>
       <c r="H22">
-        <v>5.28076</v>
+        <v>5.28136</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -950,10 +950,10 @@
         <v>0.12</v>
       </c>
       <c r="G23">
-        <v>22733422.058548633</v>
+        <v>22731537.907055005</v>
       </c>
       <c r="H23">
-        <v>5.79613</v>
+        <v>5.79683</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -991,10 +991,10 @@
         <v>0.12</v>
       </c>
       <c r="G24">
-        <v>22733422.058548633</v>
+        <v>22731537.907055005</v>
       </c>
       <c r="H24">
-        <v>5.29033</v>
+        <v>5.29096</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1114,10 +1114,10 @@
         <v>0.1</v>
       </c>
       <c r="G27">
-        <v>34637548.02</v>
+        <v>34634675.97</v>
       </c>
       <c r="H27">
-        <v>5.76677</v>
+        <v>5.76744</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1155,10 +1155,10 @@
         <v>0.1</v>
       </c>
       <c r="G28">
-        <v>34637548.02</v>
+        <v>34634675.97</v>
       </c>
       <c r="H28">
-        <v>5.24269</v>
+        <v>5.2433</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1196,10 +1196,10 @@
         <v>0.12</v>
       </c>
       <c r="G29">
-        <v>25900136.852731157</v>
+        <v>25897989.284779612</v>
       </c>
       <c r="H29">
-        <v>5.75814</v>
+        <v>5.75883</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1237,10 +1237,10 @@
         <v>0.12</v>
       </c>
       <c r="G30">
-        <v>25900136.852731157</v>
+        <v>25897989.284779612</v>
       </c>
       <c r="H30">
-        <v>5.25109</v>
+        <v>5.25173</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1360,10 +1360,10 @@
         <v>0.1</v>
       </c>
       <c r="G33">
-        <v>40686167.02</v>
+        <v>40682524.61</v>
       </c>
       <c r="H33">
-        <v>5.53597</v>
+        <v>5.53656</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1401,10 +1401,10 @@
         <v>0.1</v>
       </c>
       <c r="G34">
-        <v>40686167.02</v>
+        <v>40682524.61</v>
       </c>
       <c r="H34">
-        <v>5.03319</v>
+        <v>5.03372</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1442,10 +1442,10 @@
         <v>0.12</v>
       </c>
       <c r="G35">
-        <v>30422976.04965044</v>
+        <v>30420252.447003417</v>
       </c>
       <c r="H35">
-        <v>5.53051</v>
+        <v>5.53108</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1483,10 +1483,10 @@
         <v>0.12</v>
       </c>
       <c r="G36">
-        <v>30422976.04965044</v>
+        <v>30420252.447003417</v>
       </c>
       <c r="H36">
-        <v>5.04186</v>
+        <v>5.04239</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1565,10 +1565,10 @@
         <v>0.65</v>
       </c>
       <c r="G38">
-        <v>986645611.91</v>
+        <v>993393228.54</v>
       </c>
       <c r="H38">
-        <v>176.18672</v>
+        <v>177.39165</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1852,10 +1852,10 @@
         <v>0.35</v>
       </c>
       <c r="G45">
-        <v>117729389.51</v>
+        <v>117728277.25</v>
       </c>
       <c r="H45">
-        <v>8.97465</v>
+        <v>8.97456</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -1893,10 +1893,10 @@
         <v>0.3</v>
       </c>
       <c r="G46">
-        <v>20024174389.98</v>
+        <v>20023483086.66</v>
       </c>
       <c r="H46">
-        <v>501.92758</v>
+        <v>501.92356</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -1934,10 +1934,10 @@
         <v>0.35</v>
       </c>
       <c r="G47">
-        <v>16068398739.23945</v>
+        <v>16067844002.890318</v>
       </c>
       <c r="H47">
-        <v>460.14784</v>
+        <v>460.05086</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -1975,10 +1975,10 @@
         <v>0.3</v>
       </c>
       <c r="G48">
-        <v>20024174389.98</v>
+        <v>20023483086.66</v>
       </c>
       <c r="H48">
-        <v>716.90582</v>
+        <v>716.90007</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2016,10 +2016,10 @@
         <v>0.35</v>
       </c>
       <c r="G49">
-        <v>14973024556.010027</v>
+        <v>14972507635.742332</v>
       </c>
       <c r="H49">
-        <v>555.88848</v>
+        <v>555.8596</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3246,10 +3246,10 @@
         <v>0.25</v>
       </c>
       <c r="G79">
-        <v>64030948.67</v>
+        <v>64040274.77</v>
       </c>
       <c r="H79">
-        <v>16.56034</v>
+        <v>16.56276</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
@@ -4763,10 +4763,10 @@
         <v>0.15</v>
       </c>
       <c r="G116">
-        <v>358292066.49</v>
+        <v>357809776.41</v>
       </c>
       <c r="H116">
-        <v>5.18279</v>
+        <v>5.18131</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
@@ -4804,10 +4804,10 @@
         <v>0.2</v>
       </c>
       <c r="G117">
-        <v>267911965.07271856</v>
+        <v>267871814.64345953</v>
       </c>
       <c r="H117">
-        <v>5.08627</v>
+        <v>5.08549</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
@@ -5132,10 +5132,10 @@
         <v>0.25</v>
       </c>
       <c r="G125">
-        <v>375752711.13</v>
+        <v>375424699.26</v>
       </c>
       <c r="H125">
-        <v>7.25225</v>
+        <v>7.25321</v>
       </c>
       <c r="I125" t="inlineStr">
         <is>
@@ -5173,10 +5173,10 @@
         <v>0.25</v>
       </c>
       <c r="G126">
-        <v>375752711.13</v>
+        <v>375424699.26</v>
       </c>
       <c r="H126">
-        <v>5.78376</v>
+        <v>5.78452</v>
       </c>
       <c r="I126" t="inlineStr">
         <is>
@@ -5214,10 +5214,10 @@
         <v>0.3</v>
       </c>
       <c r="G127">
-        <v>328369056.3051645</v>
+        <v>328096743.9458171</v>
       </c>
       <c r="H127">
-        <v>6.824</v>
+        <v>6.82488</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
@@ -5255,10 +5255,10 @@
         <v>0.3</v>
       </c>
       <c r="G128">
-        <v>280968116.8953529</v>
+        <v>281059104.81751907</v>
       </c>
       <c r="H128">
-        <v>5.70818</v>
+        <v>5.70916</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
@@ -5419,10 +5419,10 @@
         <v>0.19</v>
       </c>
       <c r="G132">
-        <v>33273786765.022125</v>
+        <v>33647419275.54283</v>
       </c>
       <c r="H132">
-        <v>45711.3206</v>
+        <v>46214.1275</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
@@ -5459,8 +5459,12 @@
       <c r="F133">
         <v>0.19</v>
       </c>
-      <c r="G133"/>
-      <c r="H133"/>
+      <c r="G133">
+        <v>182321064.9009745</v>
+      </c>
+      <c r="H133">
+        <v>46.4774</v>
+      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t xml:space="preserve">[]</t>
@@ -5496,8 +5500,12 @@
       <c r="F134">
         <v>0.19</v>
       </c>
-      <c r="G134"/>
-      <c r="H134"/>
+      <c r="G134">
+        <v>208620897.22931704</v>
+      </c>
+      <c r="H134">
+        <v>57.4478</v>
+      </c>
       <c r="I134" t="inlineStr">
         <is>
           <t xml:space="preserve">[]</t>
@@ -6477,10 +6485,10 @@
         <v>0.09</v>
       </c>
       <c r="G158">
-        <v>64463199.71</v>
+        <v>64463044.87</v>
       </c>
       <c r="H158">
-        <v>6.85779</v>
+        <v>6.85777</v>
       </c>
       <c r="I158" t="inlineStr">
         <is>
@@ -6641,10 +6649,10 @@
         <v>0.09</v>
       </c>
       <c r="G162">
-        <v>3130719020.94</v>
+        <v>3149560805.61</v>
       </c>
       <c r="H162">
-        <v>114.26951</v>
+        <v>114.26926</v>
       </c>
       <c r="I162" t="inlineStr">
         <is>
@@ -6682,10 +6690,10 @@
         <v>0.09</v>
       </c>
       <c r="G163">
-        <v>3130719020.94</v>
+        <v>3149560805.61</v>
       </c>
       <c r="H163">
-        <v>107.84049</v>
+        <v>107.84025</v>
       </c>
       <c r="I163" t="inlineStr">
         <is>
@@ -6723,10 +6731,10 @@
         <v>0.12</v>
       </c>
       <c r="G164">
-        <v>2340987042.2402525</v>
+        <v>2355075937.944443</v>
       </c>
       <c r="H164">
-        <v>108.31853</v>
+        <v>108.31837</v>
       </c>
       <c r="I164" t="inlineStr">
         <is>
@@ -7092,10 +7100,10 @@
         <v>0.25</v>
       </c>
       <c r="G173">
-        <v>51159062.79</v>
+        <v>51158743.93</v>
       </c>
       <c r="H173">
-        <v>55.3071</v>
+        <v>55.30675</v>
       </c>
       <c r="I173" t="inlineStr">
         <is>
@@ -7215,10 +7223,10 @@
         <v>0.2</v>
       </c>
       <c r="G176">
-        <v>113976217</v>
+        <v>115603838.44</v>
       </c>
       <c r="H176">
-        <v>8.14116</v>
+        <v>8.14112</v>
       </c>
       <c r="I176" t="inlineStr">
         <is>
@@ -7338,10 +7346,10 @@
         <v>0.29</v>
       </c>
       <c r="G179">
-        <v>7368369.56</v>
+        <v>7370552.3</v>
       </c>
       <c r="H179">
-        <v>21.05248</v>
+        <v>21.05872</v>
       </c>
       <c r="I179" t="inlineStr">
         <is>
@@ -7675,10 +7683,10 @@
         <v>0.5</v>
       </c>
       <c r="G188">
-        <v>188052474.33</v>
+        <v>188048742.77</v>
       </c>
       <c r="H188">
-        <v>46.42928</v>
+        <v>46.42865</v>
       </c>
       <c r="I188" t="inlineStr">
         <is>
@@ -7716,10 +7724,10 @@
         <v>0.5</v>
       </c>
       <c r="G189">
-        <v>188052474.33</v>
+        <v>188048742.77</v>
       </c>
       <c r="H189">
-        <v>14.44772</v>
+        <v>14.44752</v>
       </c>
       <c r="I189" t="inlineStr">
         <is>
@@ -8003,10 +8011,10 @@
         <v>0.09</v>
       </c>
       <c r="G196">
-        <v>2472943.61</v>
+        <v>2472937.7</v>
       </c>
       <c r="H196">
-        <v>6.18236</v>
+        <v>6.18234</v>
       </c>
       <c r="I196" t="inlineStr">
         <is>
@@ -8085,10 +8093,10 @@
         <v>0.2</v>
       </c>
       <c r="G198">
-        <v>1606819111.05</v>
+        <v>1606811607.19</v>
       </c>
       <c r="H198">
-        <v>73.48344</v>
+        <v>73.48309</v>
       </c>
       <c r="I198" t="inlineStr">
         <is>
@@ -8126,10 +8134,10 @@
         <v>0.2</v>
       </c>
       <c r="G199">
-        <v>1606819111.05</v>
+        <v>1606811607.19</v>
       </c>
       <c r="H199">
-        <v>68.23427</v>
+        <v>68.23395</v>
       </c>
       <c r="I199" t="inlineStr">
         <is>
@@ -8167,10 +8175,10 @@
         <v>0.35</v>
       </c>
       <c r="G200">
-        <v>355677054.82353</v>
+        <v>355664430.1585375</v>
       </c>
       <c r="H200">
-        <v>31.98578</v>
+        <v>31.98161</v>
       </c>
       <c r="I200" t="inlineStr">
         <is>
@@ -8208,10 +8216,10 @@
         <v>0.3</v>
       </c>
       <c r="G201">
-        <v>443238899.4</v>
+        <v>443223166.75</v>
       </c>
       <c r="H201">
-        <v>38.97834</v>
+        <v>38.97805</v>
       </c>
       <c r="I201" t="inlineStr">
         <is>
@@ -8249,10 +8257,10 @@
         <v>0.25</v>
       </c>
       <c r="G202">
-        <v>139117692.66</v>
+        <v>139116751.97</v>
       </c>
       <c r="H202">
-        <v>55.64708</v>
+        <v>55.6467</v>
       </c>
       <c r="I202" t="inlineStr">
         <is>
@@ -8331,10 +8339,10 @@
         <v>0.2</v>
       </c>
       <c r="G204">
-        <v>24318430.47</v>
+        <v>24318390.18</v>
       </c>
       <c r="H204">
-        <v>6.40537</v>
+        <v>6.40536</v>
       </c>
       <c r="I204" t="inlineStr">
         <is>
@@ -8372,10 +8380,10 @@
         <v>0.2</v>
       </c>
       <c r="G205">
-        <v>24318430.47</v>
+        <v>24318390.18</v>
       </c>
       <c r="H205">
-        <v>6.34907</v>
+        <v>6.34906</v>
       </c>
       <c r="I205" t="inlineStr">
         <is>
@@ -10012,10 +10020,10 @@
         <v>0.16</v>
       </c>
       <c r="G245">
-        <v>130851428.53</v>
+        <v>130850883.13</v>
       </c>
       <c r="H245">
-        <v>5.7391</v>
+        <v>5.73907</v>
       </c>
       <c r="I245" t="inlineStr">
         <is>
@@ -10053,10 +10061,10 @@
         <v>0.45</v>
       </c>
       <c r="G246">
-        <v>89676759.58</v>
+        <v>89681545.41</v>
       </c>
       <c r="H246">
-        <v>31.96755</v>
+        <v>31.97074</v>
       </c>
       <c r="I246" t="inlineStr">
         <is>
@@ -10094,10 +10102,10 @@
         <v>0.45</v>
       </c>
       <c r="G247">
-        <v>89676759.58</v>
+        <v>89681545.41</v>
       </c>
       <c r="H247">
-        <v>21.4638</v>
+        <v>21.46594</v>
       </c>
       <c r="I247" t="inlineStr">
         <is>
@@ -10135,10 +10143,10 @@
         <v>0.5</v>
       </c>
       <c r="G248">
-        <v>67055564.79605192</v>
+        <v>67059143.388043545</v>
       </c>
       <c r="H248">
-        <v>30.81325</v>
+        <v>30.81642</v>
       </c>
       <c r="I248" t="inlineStr">
         <is>
@@ -10176,10 +10184,10 @@
         <v>0.28</v>
       </c>
       <c r="G249">
-        <v>15477791.57</v>
+        <v>15479908.69</v>
       </c>
       <c r="H249">
-        <v>31.88897</v>
+        <v>31.89334</v>
       </c>
       <c r="I249" t="inlineStr">
         <is>
@@ -10217,10 +10225,10 @@
         <v>0.06</v>
       </c>
       <c r="G250">
-        <v>609992785.84</v>
+        <v>615432775.72</v>
       </c>
       <c r="H250">
-        <v>48.50546</v>
+        <v>48.50966</v>
       </c>
       <c r="I250" t="inlineStr">
         <is>
@@ -10258,10 +10266,10 @@
         <v>0.06</v>
       </c>
       <c r="G251">
-        <v>609992785.84</v>
+        <v>615432775.72</v>
       </c>
       <c r="H251">
-        <v>40.51954</v>
+        <v>40.52305</v>
       </c>
       <c r="I251" t="inlineStr">
         <is>
@@ -10299,10 +10307,10 @@
         <v>0.1</v>
       </c>
       <c r="G252">
-        <v>533070685.8690899</v>
+        <v>537824675.1026825</v>
       </c>
       <c r="H252">
-        <v>43.67136</v>
+        <v>43.67311</v>
       </c>
       <c r="I252" t="inlineStr">
         <is>
@@ -10340,10 +10348,10 @@
         <v>0.1</v>
       </c>
       <c r="G253">
-        <v>456120526.2945379</v>
+        <v>460188264.64276385</v>
       </c>
       <c r="H253">
-        <v>39.64915</v>
+        <v>39.65275</v>
       </c>
       <c r="I253" t="inlineStr">
         <is>
@@ -10381,10 +10389,10 @@
         <v>0.1</v>
       </c>
       <c r="G254">
-        <v>10654133997.48144</v>
+        <v>10749148860.72552</v>
       </c>
       <c r="H254">
-        <v>1060.36168</v>
+        <v>1060.55089</v>
       </c>
       <c r="I254" t="inlineStr">
         <is>
@@ -10422,10 +10430,10 @@
         <v>0.06</v>
       </c>
       <c r="G255">
-        <v>302167666.87</v>
+        <v>302135518.17</v>
       </c>
       <c r="H255">
-        <v>44.10297</v>
+        <v>44.10683</v>
       </c>
       <c r="I255" t="inlineStr">
         <is>
@@ -10463,10 +10471,10 @@
         <v>0.06</v>
       </c>
       <c r="G256">
-        <v>302167666.87</v>
+        <v>302135518.17</v>
       </c>
       <c r="H256">
-        <v>38.42171</v>
+        <v>38.42507</v>
       </c>
       <c r="I256" t="inlineStr">
         <is>
@@ -10504,10 +10512,10 @@
         <v>0.1</v>
       </c>
       <c r="G257">
-        <v>264063328.55894414</v>
+        <v>264035233.91593096</v>
       </c>
       <c r="H257">
-        <v>34.56042</v>
+        <v>34.56182</v>
       </c>
       <c r="I257" t="inlineStr">
         <is>
@@ -10545,10 +10553,10 @@
         <v>0.1</v>
       </c>
       <c r="G258">
-        <v>225945090.5671665</v>
+        <v>225921051.4599769</v>
       </c>
       <c r="H258">
-        <v>36.66978</v>
+        <v>36.67323</v>
       </c>
       <c r="I258" t="inlineStr">
         <is>
@@ -10586,10 +10594,10 @@
         <v>0.06</v>
       </c>
       <c r="G259">
-        <v>187616441.04</v>
+        <v>187600829.33</v>
       </c>
       <c r="H259">
-        <v>4.80692</v>
+        <v>4.80747</v>
       </c>
       <c r="I259" t="inlineStr">
         <is>
@@ -10627,10 +10635,10 @@
         <v>0.06</v>
       </c>
       <c r="G260">
-        <v>187616441.04</v>
+        <v>187600829.33</v>
       </c>
       <c r="H260">
-        <v>4.09121</v>
+        <v>4.09168</v>
       </c>
       <c r="I260" t="inlineStr">
         <is>
@@ -10668,10 +10676,10 @@
         <v>0.1</v>
       </c>
       <c r="G261">
-        <v>163957389.7054967</v>
+        <v>163943746.6835619</v>
       </c>
       <c r="H261">
-        <v>3.76031</v>
+        <v>3.76043</v>
       </c>
       <c r="I261" t="inlineStr">
         <is>
@@ -10709,10 +10717,10 @@
         <v>0.1</v>
       </c>
       <c r="G262">
-        <v>140289708.034546</v>
+        <v>140278034.41881338</v>
       </c>
       <c r="H262">
-        <v>3.96815</v>
+        <v>3.9685</v>
       </c>
       <c r="I262" t="inlineStr">
         <is>
@@ -10750,10 +10758,10 @@
         <v>0.06</v>
       </c>
       <c r="G263">
-        <v>215238728.65</v>
+        <v>215219302.56</v>
       </c>
       <c r="H263">
-        <v>44.15382</v>
+        <v>44.15808</v>
       </c>
       <c r="I263" t="inlineStr">
         <is>
@@ -10791,10 +10799,10 @@
         <v>0.06</v>
       </c>
       <c r="G264">
-        <v>215238728.65</v>
+        <v>215219302.56</v>
       </c>
       <c r="H264">
-        <v>37.47687</v>
+        <v>37.48048</v>
       </c>
       <c r="I264" t="inlineStr">
         <is>
@@ -10832,10 +10840,10 @@
         <v>0.1</v>
       </c>
       <c r="G265">
-        <v>188096415.84374714</v>
+        <v>188079439.44769716</v>
       </c>
       <c r="H265">
-        <v>32.69347</v>
+        <v>32.69508</v>
       </c>
       <c r="I265" t="inlineStr">
         <is>
@@ -10873,10 +10881,10 @@
         <v>0.1</v>
       </c>
       <c r="G266">
-        <v>160944202.07873788</v>
+        <v>160929676.270236</v>
       </c>
       <c r="H266">
-        <v>35.53415</v>
+        <v>35.5374</v>
       </c>
       <c r="I266" t="inlineStr">
         <is>
@@ -10914,10 +10922,10 @@
         <v>0.06</v>
       </c>
       <c r="G267">
-        <v>2673639647.72</v>
+        <v>2671227151.6</v>
       </c>
       <c r="H267">
-        <v>44.07193</v>
+        <v>44.07717</v>
       </c>
       <c r="I267" t="inlineStr">
         <is>
@@ -10955,10 +10963,10 @@
         <v>0.1</v>
       </c>
       <c r="G268">
-        <v>2145462135.312914</v>
+        <v>2143526227.80142</v>
       </c>
       <c r="H268">
-        <v>39.62468</v>
+        <v>39.62369</v>
       </c>
       <c r="I268" t="inlineStr">
         <is>
@@ -10996,10 +11004,10 @@
         <v>0.06</v>
       </c>
       <c r="G269">
-        <v>2673639647.72</v>
+        <v>2671227151.6</v>
       </c>
       <c r="H269">
-        <v>35.17921</v>
+        <v>35.18339</v>
       </c>
       <c r="I269" t="inlineStr">
         <is>
@@ -11037,10 +11045,10 @@
         <v>0.1</v>
       </c>
       <c r="G270">
-        <v>2336484879.59451</v>
+        <v>2334376607.1834292</v>
       </c>
       <c r="H270">
-        <v>30.19306</v>
+        <v>30.19524</v>
       </c>
       <c r="I270" t="inlineStr">
         <is>
@@ -11078,10 +11086,10 @@
         <v>0.1</v>
       </c>
       <c r="G271">
-        <v>1999207124.3279629</v>
+        <v>1997403186.6003673</v>
       </c>
       <c r="H271">
-        <v>33.29989</v>
+        <v>33.3039</v>
       </c>
       <c r="I271" t="inlineStr">
         <is>
@@ -11119,10 +11127,10 @@
         <v>0.06</v>
       </c>
       <c r="G272">
-        <v>652067421.39</v>
+        <v>654259410.56</v>
       </c>
       <c r="H272">
-        <v>44.17133</v>
+        <v>44.17574</v>
       </c>
       <c r="I272" t="inlineStr">
         <is>
@@ -11160,10 +11168,10 @@
         <v>0.1</v>
       </c>
       <c r="G273">
-        <v>523251502.2944055</v>
+        <v>525010464.003872</v>
       </c>
       <c r="H273">
-        <v>39.31428</v>
+        <v>39.31262</v>
       </c>
       <c r="I273" t="inlineStr">
         <is>
@@ -11201,10 +11209,10 @@
         <v>0.06</v>
       </c>
       <c r="G274">
-        <v>652067421.39</v>
+        <v>654259410.56</v>
       </c>
       <c r="H274">
-        <v>35.67052</v>
+        <v>35.67408</v>
       </c>
       <c r="I274" t="inlineStr">
         <is>
@@ -11242,10 +11250,10 @@
         <v>0.1</v>
       </c>
       <c r="G275">
-        <v>569839571.257537</v>
+        <v>571755143.3714931</v>
       </c>
       <c r="H275">
-        <v>30.87045</v>
+        <v>30.87211</v>
       </c>
       <c r="I275" t="inlineStr">
         <is>
@@ -11283,10 +11291,10 @@
         <v>0.1</v>
       </c>
       <c r="G276">
-        <v>487581726.0926461</v>
+        <v>489220780.3192884</v>
       </c>
       <c r="H276">
-        <v>32.8487</v>
+        <v>32.85196</v>
       </c>
       <c r="I276" t="inlineStr">
         <is>
@@ -11324,10 +11332,10 @@
         <v>0.25</v>
       </c>
       <c r="G277">
-        <v>813767291.47</v>
+        <v>813098003.24</v>
       </c>
       <c r="H277">
-        <v>21.3739</v>
+        <v>21.37688</v>
       </c>
       <c r="I277" t="inlineStr">
         <is>
@@ -11365,10 +11373,10 @@
         <v>0.25</v>
       </c>
       <c r="G278">
-        <v>813767291.47</v>
+        <v>813098003.24</v>
       </c>
       <c r="H278">
-        <v>20.04787</v>
+        <v>20.05067</v>
       </c>
       <c r="I278" t="inlineStr">
         <is>
@@ -11406,10 +11414,10 @@
         <v>0.25</v>
       </c>
       <c r="G279">
-        <v>608492385.2918087</v>
+        <v>607991926.7506639</v>
       </c>
       <c r="H279">
-        <v>16.90886</v>
+        <v>16.91133</v>
       </c>
       <c r="I279" t="inlineStr">
         <is>
@@ -11447,10 +11455,10 @@
         <v>0.25</v>
       </c>
       <c r="G280">
-        <v>608492385.2918087</v>
+        <v>607991926.7506639</v>
       </c>
       <c r="H280">
-        <v>16.07654</v>
+        <v>16.07892</v>
       </c>
       <c r="I280" t="inlineStr">
         <is>
@@ -11488,10 +11496,10 @@
         <v>0.39</v>
       </c>
       <c r="G281">
-        <v>1660435182.03</v>
+        <v>1662239654.66</v>
       </c>
       <c r="H281">
-        <v>30.32331</v>
+        <v>30.32871</v>
       </c>
       <c r="I281" t="inlineStr">
         <is>
@@ -11529,10 +11537,10 @@
         <v>0.39</v>
       </c>
       <c r="G282">
-        <v>1660435182.03</v>
+        <v>1662239654.66</v>
       </c>
       <c r="H282">
-        <v>19.23008</v>
+        <v>19.23351</v>
       </c>
       <c r="I282" t="inlineStr">
         <is>
@@ -11570,10 +11578,10 @@
         <v>0.39</v>
       </c>
       <c r="G283">
-        <v>1451048835.1219075</v>
+        <v>1452625757.8082662</v>
       </c>
       <c r="H283">
-        <v>16.23073</v>
+        <v>16.23289</v>
       </c>
       <c r="I283" t="inlineStr">
         <is>
@@ -11611,10 +11619,10 @@
         <v>0.39</v>
       </c>
       <c r="G284">
-        <v>1241586108.3710327</v>
+        <v>1242935398.1081996</v>
       </c>
       <c r="H284">
-        <v>35.1919</v>
+        <v>35.19854</v>
       </c>
       <c r="I284" t="inlineStr">
         <is>
@@ -11652,10 +11660,10 @@
         <v>0.1</v>
       </c>
       <c r="G285">
-        <v>42043558.95</v>
+        <v>42038977.29</v>
       </c>
       <c r="H285">
-        <v>18.22124</v>
+        <v>18.22362</v>
       </c>
       <c r="I285" t="inlineStr">
         <is>
@@ -11693,10 +11701,10 @@
         <v>0.12</v>
       </c>
       <c r="G286">
-        <v>31437962.350917872</v>
+        <v>31434536.426515136</v>
       </c>
       <c r="H286">
-        <v>32.92331</v>
+        <v>32.92739</v>
       </c>
       <c r="I286" t="inlineStr">
         <is>
@@ -11734,10 +11742,10 @@
         <v>0.15</v>
       </c>
       <c r="G287">
-        <v>9856785.63</v>
+        <v>9857849.88</v>
       </c>
       <c r="H287">
-        <v>5.10524</v>
+        <v>5.10594</v>
       </c>
       <c r="I287" t="inlineStr">
         <is>
@@ -11775,10 +11783,10 @@
         <v>0.15</v>
       </c>
       <c r="G288">
-        <v>9856785.63</v>
+        <v>9857849.88</v>
       </c>
       <c r="H288">
-        <v>5.03999</v>
+        <v>5.04068</v>
       </c>
       <c r="I288" t="inlineStr">
         <is>
@@ -11816,10 +11824,10 @@
         <v>0.17</v>
       </c>
       <c r="G289">
-        <v>7370385.934871203</v>
+        <v>7371181.725053281</v>
       </c>
       <c r="H289">
-        <v>5.03863</v>
+        <v>5.03934</v>
       </c>
       <c r="I289" t="inlineStr">
         <is>
@@ -11939,10 +11947,10 @@
         <v>0.5</v>
       </c>
       <c r="G292">
-        <v>23230256.77</v>
+        <v>23233342.24</v>
       </c>
       <c r="H292">
-        <v>59.69246</v>
+        <v>59.70039</v>
       </c>
       <c r="I292" t="inlineStr">
         <is>
@@ -11980,10 +11988,10 @@
         <v>0.5</v>
       </c>
       <c r="G293">
-        <v>23230256.77</v>
+        <v>23233342.24</v>
       </c>
       <c r="H293">
-        <v>39.93199</v>
+        <v>39.93729</v>
       </c>
       <c r="I293" t="inlineStr">
         <is>

</xml_diff>